<commit_message>
Auto update and deploy
</commit_message>
<xml_diff>
--- a/hebrew-owner-review/hebrew_copy_review_master_package_WITH_SUGGESTIONS_FIXED/01_PARENT_REPORT/parent-report-hebrew-owner-review-01-rows-001-050.xlsx
+++ b/hebrew-owner-review/hebrew_copy_review_master_package_WITH_SUGGESTIONS_FIXED/01_PARENT_REPORT/parent-report-hebrew-owner-review-01-rows-001-050.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ERAN YOSEF\Desktop\final projects\FINAL-WEB\LIOSH-WEB-TRY\hebrew-owner-review\hebrew_copy_review_master_package_WITH_SUGGESTIONS_FIXED\01_PARENT_REPORT\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D4A5258-C99D-4A59-9C49-46B528EC9622}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="לאישור" sheetId="1" r:id="rId1"/>
@@ -13,12 +19,12 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">לאישור!$A$1:$K$51</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="317">
   <si>
     <t>מספר</t>
   </si>
@@ -1080,13 +1086,16 @@
   </si>
   <si>
     <t>Cursor לא מנסח לבד. הוא מיישם רק לפי אישור הבעלים.</t>
+  </si>
+  <si>
+    <t>מאושר</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1237,13 +1246,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1281,7 +1298,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -1315,6 +1332,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -1349,9 +1367,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1524,21 +1543,24 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K51"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.7109375" customWidth="1"/>
-    <col min="2" max="2" width="24.7109375" customWidth="1"/>
-    <col min="3" max="5" width="44.7109375" customWidth="1"/>
-    <col min="6" max="6" width="16.7109375" customWidth="1"/>
-    <col min="7" max="7" width="38.7109375" customWidth="1"/>
-    <col min="8" max="9" width="52.7109375" customWidth="1"/>
-    <col min="10" max="10" width="40.7109375" customWidth="1"/>
-    <col min="11" max="11" width="52.7109375" customWidth="1"/>
+    <col min="1" max="1" width="8.6640625" customWidth="1"/>
+    <col min="2" max="2" width="12.5546875" customWidth="1"/>
+    <col min="3" max="3" width="24.6640625" customWidth="1"/>
+    <col min="4" max="4" width="23.6640625" customWidth="1"/>
+    <col min="5" max="5" width="20.33203125" customWidth="1"/>
+    <col min="6" max="6" width="10.6640625" customWidth="1"/>
+    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="8" max="8" width="34.44140625" customWidth="1"/>
+    <col min="9" max="9" width="30.77734375" customWidth="1"/>
+    <col min="10" max="10" width="23.5546875" customWidth="1"/>
+    <col min="11" max="11" width="46.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="32" customHeight="1">
+    <row r="1" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1573,7 +1595,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="88" customHeight="1">
+    <row r="2" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>11</v>
       </c>
@@ -1590,7 +1612,7 @@
         <v>15</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G2" s="8" t="s">
         <v>16</v>
@@ -1608,7 +1630,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="88" customHeight="1">
+    <row r="3" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>21</v>
       </c>
@@ -1625,7 +1647,7 @@
         <v>25</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G3" s="8" t="s">
         <v>16</v>
@@ -1643,7 +1665,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="88" customHeight="1">
+    <row r="4" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>30</v>
       </c>
@@ -1660,7 +1682,7 @@
         <v>32</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G4" s="8" t="s">
         <v>16</v>
@@ -1678,7 +1700,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="88" customHeight="1">
+    <row r="5" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>37</v>
       </c>
@@ -1695,7 +1717,7 @@
         <v>41</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G5" s="8" t="s">
         <v>16</v>
@@ -1713,7 +1735,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="88" customHeight="1">
+    <row r="6" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>46</v>
       </c>
@@ -1730,7 +1752,7 @@
         <v>50</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G6" s="8" t="s">
         <v>16</v>
@@ -1748,7 +1770,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="88" customHeight="1">
+    <row r="7" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>55</v>
       </c>
@@ -1765,7 +1787,7 @@
         <v>58</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G7" s="8" t="s">
         <v>16</v>
@@ -1783,7 +1805,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="88" customHeight="1">
+    <row r="8" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>63</v>
       </c>
@@ -1800,7 +1822,7 @@
         <v>25</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G8" s="8" t="s">
         <v>16</v>
@@ -1818,7 +1840,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="88" customHeight="1">
+    <row r="9" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>68</v>
       </c>
@@ -1835,7 +1857,7 @@
         <v>70</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G9" s="8" t="s">
         <v>16</v>
@@ -1853,7 +1875,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="88" customHeight="1">
+    <row r="10" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>75</v>
       </c>
@@ -1870,7 +1892,7 @@
         <v>77</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G10" s="8" t="s">
         <v>16</v>
@@ -1888,7 +1910,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="88" customHeight="1">
+    <row r="11" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>82</v>
       </c>
@@ -1905,7 +1927,7 @@
         <v>84</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G11" s="8" t="s">
         <v>16</v>
@@ -1923,7 +1945,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="88" customHeight="1">
+    <row r="12" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>88</v>
       </c>
@@ -1940,7 +1962,7 @@
         <v>90</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G12" s="8" t="s">
         <v>16</v>
@@ -1958,7 +1980,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="88" customHeight="1">
+    <row r="13" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>94</v>
       </c>
@@ -1975,7 +1997,7 @@
         <v>96</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G13" s="8" t="s">
         <v>16</v>
@@ -1993,7 +2015,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="88" customHeight="1">
+    <row r="14" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>100</v>
       </c>
@@ -2010,7 +2032,7 @@
         <v>101</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G14" s="8" t="s">
         <v>16</v>
@@ -2028,7 +2050,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="88" customHeight="1">
+    <row r="15" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>107</v>
       </c>
@@ -2045,7 +2067,7 @@
         <v>109</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G15" s="8" t="s">
         <v>16</v>
@@ -2063,7 +2085,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="88" customHeight="1">
+    <row r="16" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>113</v>
       </c>
@@ -2080,7 +2102,7 @@
         <v>116</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G16" s="8" t="s">
         <v>16</v>
@@ -2098,7 +2120,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="88" customHeight="1">
+    <row r="17" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>120</v>
       </c>
@@ -2115,7 +2137,7 @@
         <v>122</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G17" s="8" t="s">
         <v>16</v>
@@ -2133,7 +2155,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="88" customHeight="1">
+    <row r="18" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>126</v>
       </c>
@@ -2150,7 +2172,7 @@
         <v>127</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G18" s="8" t="s">
         <v>16</v>
@@ -2168,7 +2190,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="88" customHeight="1">
+    <row r="19" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>131</v>
       </c>
@@ -2185,7 +2207,7 @@
         <v>132</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G19" s="8" t="s">
         <v>16</v>
@@ -2203,7 +2225,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="88" customHeight="1">
+    <row r="20" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>138</v>
       </c>
@@ -2220,7 +2242,7 @@
         <v>139</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G20" s="8" t="s">
         <v>16</v>
@@ -2238,7 +2260,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="88" customHeight="1">
+    <row r="21" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>144</v>
       </c>
@@ -2255,7 +2277,7 @@
         <v>145</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G21" s="8" t="s">
         <v>16</v>
@@ -2273,7 +2295,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="88" customHeight="1">
+    <row r="22" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>149</v>
       </c>
@@ -2290,7 +2312,7 @@
         <v>150</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G22" s="8" t="s">
         <v>16</v>
@@ -2308,7 +2330,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="88" customHeight="1">
+    <row r="23" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>154</v>
       </c>
@@ -2325,7 +2347,7 @@
         <v>155</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G23" s="8" t="s">
         <v>16</v>
@@ -2343,7 +2365,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="88" customHeight="1">
+    <row r="24" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>159</v>
       </c>
@@ -2360,7 +2382,7 @@
         <v>160</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G24" s="8" t="s">
         <v>16</v>
@@ -2378,7 +2400,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="88" customHeight="1">
+    <row r="25" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>164</v>
       </c>
@@ -2395,7 +2417,7 @@
         <v>165</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G25" s="8" t="s">
         <v>16</v>
@@ -2413,7 +2435,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="88" customHeight="1">
+    <row r="26" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>169</v>
       </c>
@@ -2430,7 +2452,7 @@
         <v>170</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G26" s="8" t="s">
         <v>16</v>
@@ -2448,7 +2470,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="88" customHeight="1">
+    <row r="27" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>174</v>
       </c>
@@ -2465,7 +2487,7 @@
         <v>176</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G27" s="8" t="s">
         <v>16</v>
@@ -2483,7 +2505,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="88" customHeight="1">
+    <row r="28" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>180</v>
       </c>
@@ -2500,7 +2522,7 @@
         <v>182</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G28" s="8" t="s">
         <v>16</v>
@@ -2518,7 +2540,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="88" customHeight="1">
+    <row r="29" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>186</v>
       </c>
@@ -2535,7 +2557,7 @@
         <v>188</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G29" s="8" t="s">
         <v>16</v>
@@ -2553,7 +2575,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="88" customHeight="1">
+    <row r="30" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>192</v>
       </c>
@@ -2570,7 +2592,7 @@
         <v>194</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G30" s="8" t="s">
         <v>16</v>
@@ -2588,7 +2610,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="88" customHeight="1">
+    <row r="31" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>198</v>
       </c>
@@ -2605,7 +2627,7 @@
         <v>200</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G31" s="8" t="s">
         <v>16</v>
@@ -2623,7 +2645,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="88" customHeight="1">
+    <row r="32" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>204</v>
       </c>
@@ -2640,7 +2662,7 @@
         <v>206</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G32" s="8" t="s">
         <v>16</v>
@@ -2658,7 +2680,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="88" customHeight="1">
+    <row r="33" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>210</v>
       </c>
@@ -2675,7 +2697,7 @@
         <v>212</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G33" s="8" t="s">
         <v>16</v>
@@ -2693,7 +2715,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="88" customHeight="1">
+    <row r="34" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>216</v>
       </c>
@@ -2710,7 +2732,7 @@
         <v>217</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G34" s="8" t="s">
         <v>16</v>
@@ -2728,7 +2750,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="88" customHeight="1">
+    <row r="35" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>221</v>
       </c>
@@ -2745,7 +2767,7 @@
         <v>223</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G35" s="8" t="s">
         <v>16</v>
@@ -2763,7 +2785,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="88" customHeight="1">
+    <row r="36" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>227</v>
       </c>
@@ -2780,7 +2802,7 @@
         <v>229</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G36" s="8" t="s">
         <v>16</v>
@@ -2798,7 +2820,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="88" customHeight="1">
+    <row r="37" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>233</v>
       </c>
@@ -2815,7 +2837,7 @@
         <v>234</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G37" s="8" t="s">
         <v>16</v>
@@ -2833,7 +2855,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="38" spans="1:11" ht="88" customHeight="1">
+    <row r="38" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>238</v>
       </c>
@@ -2850,7 +2872,7 @@
         <v>239</v>
       </c>
       <c r="F38" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G38" s="8" t="s">
         <v>16</v>
@@ -2868,7 +2890,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="88" customHeight="1">
+    <row r="39" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>243</v>
       </c>
@@ -2885,7 +2907,7 @@
         <v>244</v>
       </c>
       <c r="F39" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G39" s="8" t="s">
         <v>16</v>
@@ -2903,7 +2925,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="40" spans="1:11" ht="88" customHeight="1">
+    <row r="40" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>248</v>
       </c>
@@ -2920,7 +2942,7 @@
         <v>249</v>
       </c>
       <c r="F40" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G40" s="8" t="s">
         <v>16</v>
@@ -2938,7 +2960,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="88" customHeight="1">
+    <row r="41" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>253</v>
       </c>
@@ -2955,7 +2977,7 @@
         <v>254</v>
       </c>
       <c r="F41" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G41" s="8" t="s">
         <v>16</v>
@@ -2973,7 +2995,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="42" spans="1:11" ht="88" customHeight="1">
+    <row r="42" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>258</v>
       </c>
@@ -2990,7 +3012,7 @@
         <v>259</v>
       </c>
       <c r="F42" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G42" s="8" t="s">
         <v>16</v>
@@ -3008,7 +3030,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="88" customHeight="1">
+    <row r="43" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>263</v>
       </c>
@@ -3025,7 +3047,7 @@
         <v>264</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G43" s="8" t="s">
         <v>16</v>
@@ -3043,7 +3065,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="44" spans="1:11" ht="88" customHeight="1">
+    <row r="44" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>268</v>
       </c>
@@ -3060,7 +3082,7 @@
         <v>269</v>
       </c>
       <c r="F44" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G44" s="8" t="s">
         <v>16</v>
@@ -3078,7 +3100,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="45" spans="1:11" ht="88" customHeight="1">
+    <row r="45" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>273</v>
       </c>
@@ -3095,7 +3117,7 @@
         <v>274</v>
       </c>
       <c r="F45" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G45" s="8" t="s">
         <v>16</v>
@@ -3113,7 +3135,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="88" customHeight="1">
+    <row r="46" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>278</v>
       </c>
@@ -3130,7 +3152,7 @@
         <v>279</v>
       </c>
       <c r="F46" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G46" s="8" t="s">
         <v>16</v>
@@ -3148,7 +3170,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="47" spans="1:11" ht="88" customHeight="1">
+    <row r="47" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>283</v>
       </c>
@@ -3165,7 +3187,7 @@
         <v>284</v>
       </c>
       <c r="F47" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G47" s="8" t="s">
         <v>16</v>
@@ -3183,7 +3205,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="48" spans="1:11" ht="88" customHeight="1">
+    <row r="48" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>288</v>
       </c>
@@ -3200,7 +3222,7 @@
         <v>290</v>
       </c>
       <c r="F48" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G48" s="8" t="s">
         <v>16</v>
@@ -3218,7 +3240,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="49" spans="1:11" ht="88" customHeight="1">
+    <row r="49" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>294</v>
       </c>
@@ -3235,7 +3257,7 @@
         <v>296</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G49" s="8" t="s">
         <v>16</v>
@@ -3253,7 +3275,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="50" spans="1:11" ht="88" customHeight="1">
+    <row r="50" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>300</v>
       </c>
@@ -3270,7 +3292,7 @@
         <v>301</v>
       </c>
       <c r="F50" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G50" s="8" t="s">
         <v>16</v>
@@ -3288,7 +3310,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="51" spans="1:11" ht="88" customHeight="1">
+    <row r="51" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>305</v>
       </c>
@@ -3305,7 +3327,7 @@
         <v>306</v>
       </c>
       <c r="F51" s="7" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="G51" s="8" t="s">
         <v>16</v>
@@ -3324,9 +3346,9 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K51"/>
+  <autoFilter ref="A1:K51" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F51">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F51" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"מאושר,לשנות,לא בטוח"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3335,39 +3357,39 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="110.7109375" customWidth="1"/>
+    <col min="1" max="1" width="110.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>310</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="3" spans="1:1">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="4" spans="1:1">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="5" spans="1:1">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="6" spans="1:1">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>315</v>
       </c>

</xml_diff>